<commit_message>
Update docs and track large epub file with LFS
</commit_message>
<xml_diff>
--- a/Hardware/Assembly/BoM.xlsx
+++ b/Hardware/Assembly/BoM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dexterous Hand\My_Bionic_hand_project\Hardware\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Bionic_hand\My_Bionic_hand_project\Hardware\Assembly\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C0D4A77-BBB8-482F-8C2A-4CAF1874511B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F7EB070-5903-49A6-A48B-C846859F2BE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4155" yWindow="1155" windowWidth="22620" windowHeight="13530" xr2:uid="{AD7F9805-AA71-4FA9-80C9-D9559D35F51B}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{AD7F9805-AA71-4FA9-80C9-D9559D35F51B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,61 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="51">
-  <si>
-    <t>类别</t>
-  </si>
-  <si>
-    <t>物品名称</t>
-  </si>
-  <si>
-    <t>数量</t>
-  </si>
-  <si>
-    <t>单价(RMB)</t>
-  </si>
-  <si>
-    <t>总共</t>
-  </si>
-  <si>
-    <t>核心电子件</t>
-  </si>
-  <si>
-    <t>AD8232传感器套件</t>
-  </si>
-  <si>
-    <t>ESP32 开发板</t>
-  </si>
-  <si>
-    <t>连接线材</t>
-  </si>
-  <si>
-    <t>杜邦线组合包</t>
-  </si>
-  <si>
-    <t>Micro-USB 数据线</t>
-  </si>
-  <si>
-    <t>面包板(400)</t>
-  </si>
-  <si>
-    <t>数字万用表</t>
-  </si>
-  <si>
-    <t>电烙铁套装</t>
-  </si>
-  <si>
-    <t>重要耗材</t>
-  </si>
-  <si>
-    <t>一次性电极片</t>
-  </si>
-  <si>
-    <t>电子元件</t>
-  </si>
-  <si>
-    <t>电阻包(套）</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
   <si>
     <t>Finger Distal/Medial and Thumb Proximal/Distal Return Spring (PIP)</t>
   </si>
@@ -98,12 +44,6 @@
     <t>Thumb CMC/MCP Return Spring (CMC)</t>
   </si>
   <si>
-    <t>绳键</t>
-  </si>
-  <si>
-    <t>耐磨抗切高分子绳 1.2mm</t>
-  </si>
-  <si>
     <t>Finger Pull Cable</t>
   </si>
   <si>
@@ -158,9 +98,6 @@
     <t>M3x5.7 Heat set insert</t>
   </si>
   <si>
-    <t>舵机一套</t>
-  </si>
-  <si>
     <t>Feetech HLS3606M Servo Motor</t>
   </si>
   <si>
@@ -182,10 +119,55 @@
     <t>ESP32-S3</t>
   </si>
   <si>
-    <t>电源适配器</t>
-  </si>
-  <si>
-    <t>总共(RMB)</t>
+    <t>SICHIRAY sEMG sets</t>
+  </si>
+  <si>
+    <t>Total(RMB)</t>
+  </si>
+  <si>
+    <t>Power adapter</t>
+  </si>
+  <si>
+    <t>A set of servos</t>
+  </si>
+  <si>
+    <t>Tether</t>
+  </si>
+  <si>
+    <t>Wear-resistant and cut-resistant polymer rope &lt;=1.2mm</t>
+  </si>
+  <si>
+    <t>Disposable electrode patch</t>
+  </si>
+  <si>
+    <t>Breadboard(400)</t>
+  </si>
+  <si>
+    <t>Micro-USB Data cable</t>
+  </si>
+  <si>
+    <t>DuPont wire bundle</t>
+  </si>
+  <si>
+    <t>ESP32 Development board</t>
+  </si>
+  <si>
+    <t>AD8232 Sensor kit</t>
+  </si>
+  <si>
+    <t>Number</t>
+  </si>
+  <si>
+    <t>unit price(RMB)</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Item Name</t>
+  </si>
+  <si>
+    <t>Categories</t>
   </si>
 </sst>
 </file>
@@ -383,12 +365,15 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFont="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="18">
     <cellStyle name="Accent" xfId="7" xr:uid="{72230192-DDDD-4147-9412-F9F06B620881}"/>
@@ -740,41 +725,39 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5618261-9B69-4922-ACFD-5100BC87D651}">
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.375" customWidth="1"/>
     <col min="2" max="2" width="44.375" style="1" customWidth="1"/>
     <col min="3" max="3" width="9.5" customWidth="1"/>
-    <col min="4" max="5" width="11.75" customWidth="1"/>
+    <col min="4" max="4" width="10.375" customWidth="1"/>
+    <col min="5" max="5" width="11.75" customWidth="1"/>
     <col min="6" max="6" width="29.375" customWidth="1"/>
     <col min="7" max="1024" width="11.75" customWidth="1"/>
     <col min="1025" max="1025" width="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>43</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
+        <v>40</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="E1" t="s">
-        <v>4</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
       <c r="B2" s="1" t="s">
-        <v>6</v>
+        <v>39</v>
       </c>
       <c r="C2">
         <v>2</v>
@@ -783,230 +766,174 @@
         <v>69.599999999999994</v>
       </c>
       <c r="E2">
-        <f t="shared" ref="E2:E40" si="0">C2*D2</f>
+        <f t="shared" ref="E2:E41" si="0">C2*D2</f>
         <v>139.19999999999999</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
       <c r="B3" s="1" t="s">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D3">
+        <v>95</v>
+      </c>
+      <c r="E3">
+        <f t="shared" si="0"/>
+        <v>190</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="B4" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
         <v>20</v>
       </c>
-      <c r="E3">
+      <c r="E4">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="D4">
+    <row r="5" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="B5" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
         <v>12</v>
       </c>
-      <c r="E4">
+      <c r="E5">
         <f t="shared" si="0"/>
         <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5">
-        <v>8.61</v>
-      </c>
-      <c r="E5">
-        <f t="shared" si="0"/>
-        <v>8.61</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
       <c r="B6" s="1" t="s">
-        <v>11</v>
+        <v>36</v>
       </c>
       <c r="C6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D6">
-        <v>15</v>
+        <v>8.61</v>
       </c>
       <c r="E6">
         <f t="shared" si="0"/>
-        <v>30</v>
+        <v>8.61</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
       <c r="B7" s="1" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="C7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D7">
-        <v>52.83</v>
+        <v>15</v>
       </c>
       <c r="E7">
         <f t="shared" si="0"/>
-        <v>52.83</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="B8" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C8">
-        <v>1</v>
-      </c>
-      <c r="D8">
-        <v>25</v>
-      </c>
-      <c r="E8">
-        <f t="shared" si="0"/>
-        <v>25</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C9">
-        <v>1</v>
-      </c>
-      <c r="D9">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="14.25" x14ac:dyDescent="0.2"/>
+    <row r="9" spans="1:5" ht="14.25" x14ac:dyDescent="0.2"/>
+    <row r="10" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="B10" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10">
         <v>28.8</v>
       </c>
-      <c r="E9">
+      <c r="E10">
         <f t="shared" si="0"/>
         <v>28.8</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10">
-        <v>1</v>
-      </c>
-      <c r="D10">
-        <v>42.56</v>
-      </c>
-      <c r="E10">
-        <f t="shared" si="0"/>
-        <v>42.56</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="28.5" x14ac:dyDescent="0.2">
-      <c r="B11" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C11">
+    <row r="11" spans="1:5" ht="14.25" x14ac:dyDescent="0.2"/>
+    <row r="12" spans="1:5" ht="28.5" x14ac:dyDescent="0.2">
+      <c r="B12" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C12">
         <v>5</v>
       </c>
-      <c r="D11">
+      <c r="D12">
         <v>2.88</v>
       </c>
-      <c r="E11">
+      <c r="E12">
         <f t="shared" si="0"/>
         <v>14.399999999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="B12" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C12">
+    <row r="13" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="B13" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C13">
         <v>4</v>
       </c>
-      <c r="D12">
+      <c r="D13">
         <v>3.6</v>
       </c>
-      <c r="E12">
+      <c r="E13">
         <f t="shared" si="0"/>
         <v>14.4</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C13">
-        <v>1</v>
-      </c>
-      <c r="D13">
+    <row r="14" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B14" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C14">
+        <v>1</v>
+      </c>
+      <c r="D14">
         <v>5.4</v>
       </c>
-      <c r="E13">
+      <c r="E14">
         <f t="shared" si="0"/>
         <v>5.4</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C14">
-        <v>1</v>
-      </c>
-      <c r="D14">
+    <row r="15" spans="1:5" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C15">
+        <v>1</v>
+      </c>
+      <c r="D15">
         <v>30.8</v>
       </c>
-      <c r="E14">
+      <c r="E15">
         <f t="shared" si="0"/>
         <v>30.8</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="2"/>
-      <c r="B15" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C15">
-        <v>3</v>
-      </c>
-      <c r="E15">
-        <f t="shared" si="0"/>
-        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2"/>
       <c r="B16" s="1" t="s">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="C16">
-        <v>1</v>
-      </c>
-      <c r="D16" s="1"/>
+        <v>3</v>
+      </c>
       <c r="E16">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1015,11 +942,12 @@
     <row r="17" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="2"/>
       <c r="B17" s="1" t="s">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="C17">
-        <v>4</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="D17" s="1"/>
       <c r="E17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1028,10 +956,10 @@
     <row r="18" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="2"/>
       <c r="B18" s="1" t="s">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="C18">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E18">
         <f t="shared" si="0"/>
@@ -1041,7 +969,7 @@
     <row r="19" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="2"/>
       <c r="B19" s="1" t="s">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="C19">
         <v>1</v>
@@ -1054,7 +982,7 @@
     <row r="20" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="2"/>
       <c r="B20" s="1" t="s">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="C20">
         <v>1</v>
@@ -1065,39 +993,40 @@
       </c>
     </row>
     <row r="21" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="2"/>
       <c r="B21" s="1" t="s">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="C21">
+        <v>1</v>
+      </c>
+      <c r="E21">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B22" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C22">
         <f>16+5</f>
         <v>21</v>
       </c>
-      <c r="D21">
+      <c r="D22">
         <v>1.5</v>
       </c>
-      <c r="E21">
+      <c r="E22">
         <f t="shared" si="0"/>
         <v>31.5</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C22">
-        <v>16</v>
-      </c>
-      <c r="E22">
-        <f t="shared" si="0"/>
-        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B23" s="1" t="s">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="C23">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="E23">
         <f t="shared" si="0"/>
@@ -1106,10 +1035,10 @@
     </row>
     <row r="24" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="1" t="s">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="C24">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="E24">
         <f t="shared" si="0"/>
@@ -1118,10 +1047,10 @@
     </row>
     <row r="25" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="1" t="s">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="C25">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="E25">
         <f t="shared" si="0"/>
@@ -1130,24 +1059,24 @@
     </row>
     <row r="26" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="1" t="s">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="C26">
+        <v>2</v>
+      </c>
+      <c r="E26">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B27" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C27">
         <f>16+5+1</f>
         <v>22</v>
       </c>
-      <c r="E26">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B27" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="C27">
-        <v>1</v>
-      </c>
       <c r="E27">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1155,7 +1084,7 @@
     </row>
     <row r="28" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="1" t="s">
-        <v>36</v>
+        <v>15</v>
       </c>
       <c r="C28">
         <v>1</v>
@@ -1167,10 +1096,10 @@
     </row>
     <row r="29" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="1" t="s">
-        <v>37</v>
+        <v>16</v>
       </c>
       <c r="C29">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="E29">
         <f t="shared" si="0"/>
@@ -1179,10 +1108,10 @@
     </row>
     <row r="30" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="1" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="C30">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="E30">
         <f t="shared" si="0"/>
@@ -1191,10 +1120,10 @@
     </row>
     <row r="31" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B31" s="1" t="s">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="C31">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E31">
         <f t="shared" si="0"/>
@@ -1203,51 +1132,53 @@
     </row>
     <row r="32" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B32" s="1" t="s">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="C32">
+        <v>9</v>
+      </c>
+      <c r="E32">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B33" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C33">
         <v>4</v>
       </c>
-      <c r="D32">
+      <c r="D33">
         <v>0.40749999999999997</v>
       </c>
-      <c r="E32">
+      <c r="E33">
         <f t="shared" si="0"/>
         <v>1.63</v>
       </c>
     </row>
-    <row r="33" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="C33">
+    <row r="34" spans="1:5" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C34">
         <v>7</v>
       </c>
-      <c r="D33">
+      <c r="D34">
         <v>345.15</v>
       </c>
-      <c r="E33">
+      <c r="E34">
         <f t="shared" si="0"/>
         <v>2416.0499999999997</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="2"/>
-      <c r="B34" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E34">
-        <f t="shared" si="0"/>
-        <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="2"/>
       <c r="B35" s="1" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="E35">
         <f t="shared" si="0"/>
@@ -1257,7 +1188,7 @@
     <row r="36" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="2"/>
       <c r="B36" s="1" t="s">
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="E36">
         <f t="shared" si="0"/>
@@ -1267,7 +1198,7 @@
     <row r="37" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="2"/>
       <c r="B37" s="1" t="s">
-        <v>46</v>
+        <v>24</v>
       </c>
       <c r="E37">
         <f t="shared" si="0"/>
@@ -1275,8 +1206,9 @@
       </c>
     </row>
     <row r="38" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="2"/>
       <c r="B38" s="1" t="s">
-        <v>47</v>
+        <v>25</v>
       </c>
       <c r="E38">
         <f t="shared" si="0"/>
@@ -1285,41 +1217,50 @@
     </row>
     <row r="39" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B39" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="C39">
-        <v>1</v>
-      </c>
-      <c r="D39">
-        <v>33.4</v>
+        <v>26</v>
       </c>
       <c r="E39">
         <f t="shared" si="0"/>
-        <v>33.4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B40" s="1" t="s">
-        <v>49</v>
+        <v>27</v>
       </c>
       <c r="C40">
         <v>1</v>
       </c>
       <c r="D40">
+        <v>33.4</v>
+      </c>
+      <c r="E40">
+        <f t="shared" si="0"/>
+        <v>33.4</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B41" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C41">
+        <v>1</v>
+      </c>
+      <c r="D41">
         <v>52</v>
       </c>
-      <c r="E40">
+      <c r="E41">
         <f t="shared" si="0"/>
         <v>52</v>
       </c>
     </row>
-    <row r="42" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D42" t="s">
-        <v>50</v>
-      </c>
-      <c r="E42">
-        <f>SUM(E2:E40)</f>
-        <v>2958.58</v>
+    <row r="45" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D45" t="s">
+        <v>29</v>
+      </c>
+      <c r="E45">
+        <f>SUM(E2:E41)</f>
+        <v>3028.1899999999996</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update docs and track large epub file with LFS (#7)
</commit_message>
<xml_diff>
--- a/Hardware/Assembly/BoM.xlsx
+++ b/Hardware/Assembly/BoM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Dexterous Hand\My_Bionic_hand_project\Hardware\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Bionic_hand\My_Bionic_hand_project\Hardware\Assembly\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C0D4A77-BBB8-482F-8C2A-4CAF1874511B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F7EB070-5903-49A6-A48B-C846859F2BE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4155" yWindow="1155" windowWidth="22620" windowHeight="13530" xr2:uid="{AD7F9805-AA71-4FA9-80C9-D9559D35F51B}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{AD7F9805-AA71-4FA9-80C9-D9559D35F51B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,61 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="51">
-  <si>
-    <t>类别</t>
-  </si>
-  <si>
-    <t>物品名称</t>
-  </si>
-  <si>
-    <t>数量</t>
-  </si>
-  <si>
-    <t>单价(RMB)</t>
-  </si>
-  <si>
-    <t>总共</t>
-  </si>
-  <si>
-    <t>核心电子件</t>
-  </si>
-  <si>
-    <t>AD8232传感器套件</t>
-  </si>
-  <si>
-    <t>ESP32 开发板</t>
-  </si>
-  <si>
-    <t>连接线材</t>
-  </si>
-  <si>
-    <t>杜邦线组合包</t>
-  </si>
-  <si>
-    <t>Micro-USB 数据线</t>
-  </si>
-  <si>
-    <t>面包板(400)</t>
-  </si>
-  <si>
-    <t>数字万用表</t>
-  </si>
-  <si>
-    <t>电烙铁套装</t>
-  </si>
-  <si>
-    <t>重要耗材</t>
-  </si>
-  <si>
-    <t>一次性电极片</t>
-  </si>
-  <si>
-    <t>电子元件</t>
-  </si>
-  <si>
-    <t>电阻包(套）</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
   <si>
     <t>Finger Distal/Medial and Thumb Proximal/Distal Return Spring (PIP)</t>
   </si>
@@ -98,12 +44,6 @@
     <t>Thumb CMC/MCP Return Spring (CMC)</t>
   </si>
   <si>
-    <t>绳键</t>
-  </si>
-  <si>
-    <t>耐磨抗切高分子绳 1.2mm</t>
-  </si>
-  <si>
     <t>Finger Pull Cable</t>
   </si>
   <si>
@@ -158,9 +98,6 @@
     <t>M3x5.7 Heat set insert</t>
   </si>
   <si>
-    <t>舵机一套</t>
-  </si>
-  <si>
     <t>Feetech HLS3606M Servo Motor</t>
   </si>
   <si>
@@ -182,10 +119,55 @@
     <t>ESP32-S3</t>
   </si>
   <si>
-    <t>电源适配器</t>
-  </si>
-  <si>
-    <t>总共(RMB)</t>
+    <t>SICHIRAY sEMG sets</t>
+  </si>
+  <si>
+    <t>Total(RMB)</t>
+  </si>
+  <si>
+    <t>Power adapter</t>
+  </si>
+  <si>
+    <t>A set of servos</t>
+  </si>
+  <si>
+    <t>Tether</t>
+  </si>
+  <si>
+    <t>Wear-resistant and cut-resistant polymer rope &lt;=1.2mm</t>
+  </si>
+  <si>
+    <t>Disposable electrode patch</t>
+  </si>
+  <si>
+    <t>Breadboard(400)</t>
+  </si>
+  <si>
+    <t>Micro-USB Data cable</t>
+  </si>
+  <si>
+    <t>DuPont wire bundle</t>
+  </si>
+  <si>
+    <t>ESP32 Development board</t>
+  </si>
+  <si>
+    <t>AD8232 Sensor kit</t>
+  </si>
+  <si>
+    <t>Number</t>
+  </si>
+  <si>
+    <t>unit price(RMB)</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>Item Name</t>
+  </si>
+  <si>
+    <t>Categories</t>
   </si>
 </sst>
 </file>
@@ -383,12 +365,15 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFont="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="18">
     <cellStyle name="Accent" xfId="7" xr:uid="{72230192-DDDD-4147-9412-F9F06B620881}"/>
@@ -740,41 +725,39 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5618261-9B69-4922-ACFD-5100BC87D651}">
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.375" customWidth="1"/>
     <col min="2" max="2" width="44.375" style="1" customWidth="1"/>
     <col min="3" max="3" width="9.5" customWidth="1"/>
-    <col min="4" max="5" width="11.75" customWidth="1"/>
+    <col min="4" max="4" width="10.375" customWidth="1"/>
+    <col min="5" max="5" width="11.75" customWidth="1"/>
     <col min="6" max="6" width="29.375" customWidth="1"/>
     <col min="7" max="1024" width="11.75" customWidth="1"/>
     <col min="1025" max="1025" width="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>43</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" t="s">
-        <v>3</v>
+        <v>40</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="E1" t="s">
-        <v>4</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
       <c r="B2" s="1" t="s">
-        <v>6</v>
+        <v>39</v>
       </c>
       <c r="C2">
         <v>2</v>
@@ -783,230 +766,174 @@
         <v>69.599999999999994</v>
       </c>
       <c r="E2">
-        <f t="shared" ref="E2:E40" si="0">C2*D2</f>
+        <f t="shared" ref="E2:E41" si="0">C2*D2</f>
         <v>139.19999999999999</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>5</v>
-      </c>
       <c r="B3" s="1" t="s">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D3">
+        <v>95</v>
+      </c>
+      <c r="E3">
+        <f t="shared" si="0"/>
+        <v>190</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="B4" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4">
+        <v>1</v>
+      </c>
+      <c r="D4">
         <v>20</v>
       </c>
-      <c r="E3">
+      <c r="E4">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4">
-        <v>1</v>
-      </c>
-      <c r="D4">
+    <row r="5" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="B5" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C5">
+        <v>1</v>
+      </c>
+      <c r="D5">
         <v>12</v>
       </c>
-      <c r="E4">
+      <c r="E5">
         <f t="shared" si="0"/>
         <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5">
-        <v>1</v>
-      </c>
-      <c r="D5">
-        <v>8.61</v>
-      </c>
-      <c r="E5">
-        <f t="shared" si="0"/>
-        <v>8.61</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
       <c r="B6" s="1" t="s">
-        <v>11</v>
+        <v>36</v>
       </c>
       <c r="C6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D6">
-        <v>15</v>
+        <v>8.61</v>
       </c>
       <c r="E6">
         <f t="shared" si="0"/>
-        <v>30</v>
+        <v>8.61</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
       <c r="B7" s="1" t="s">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="C7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D7">
-        <v>52.83</v>
+        <v>15</v>
       </c>
       <c r="E7">
         <f t="shared" si="0"/>
-        <v>52.83</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="B8" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C8">
-        <v>1</v>
-      </c>
-      <c r="D8">
-        <v>25</v>
-      </c>
-      <c r="E8">
-        <f t="shared" si="0"/>
-        <v>25</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C9">
-        <v>1</v>
-      </c>
-      <c r="D9">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="14.25" x14ac:dyDescent="0.2"/>
+    <row r="9" spans="1:5" ht="14.25" x14ac:dyDescent="0.2"/>
+    <row r="10" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="B10" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+      <c r="D10">
         <v>28.8</v>
       </c>
-      <c r="E9">
+      <c r="E10">
         <f t="shared" si="0"/>
         <v>28.8</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C10">
-        <v>1</v>
-      </c>
-      <c r="D10">
-        <v>42.56</v>
-      </c>
-      <c r="E10">
-        <f t="shared" si="0"/>
-        <v>42.56</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="28.5" x14ac:dyDescent="0.2">
-      <c r="B11" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C11">
+    <row r="11" spans="1:5" ht="14.25" x14ac:dyDescent="0.2"/>
+    <row r="12" spans="1:5" ht="28.5" x14ac:dyDescent="0.2">
+      <c r="B12" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C12">
         <v>5</v>
       </c>
-      <c r="D11">
+      <c r="D12">
         <v>2.88</v>
       </c>
-      <c r="E11">
+      <c r="E12">
         <f t="shared" si="0"/>
         <v>14.399999999999999</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="B12" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C12">
+    <row r="13" spans="1:5" ht="14.25" x14ac:dyDescent="0.2">
+      <c r="B13" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C13">
         <v>4</v>
       </c>
-      <c r="D12">
+      <c r="D13">
         <v>3.6</v>
       </c>
-      <c r="E12">
+      <c r="E13">
         <f t="shared" si="0"/>
         <v>14.4</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C13">
-        <v>1</v>
-      </c>
-      <c r="D13">
+    <row r="14" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B14" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C14">
+        <v>1</v>
+      </c>
+      <c r="D14">
         <v>5.4</v>
       </c>
-      <c r="E13">
+      <c r="E14">
         <f t="shared" si="0"/>
         <v>5.4</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C14">
-        <v>1</v>
-      </c>
-      <c r="D14">
+    <row r="15" spans="1:5" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C15">
+        <v>1</v>
+      </c>
+      <c r="D15">
         <v>30.8</v>
       </c>
-      <c r="E14">
+      <c r="E15">
         <f t="shared" si="0"/>
         <v>30.8</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="2"/>
-      <c r="B15" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C15">
-        <v>3</v>
-      </c>
-      <c r="E15">
-        <f t="shared" si="0"/>
-        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="2"/>
       <c r="B16" s="1" t="s">
-        <v>24</v>
+        <v>3</v>
       </c>
       <c r="C16">
-        <v>1</v>
-      </c>
-      <c r="D16" s="1"/>
+        <v>3</v>
+      </c>
       <c r="E16">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1015,11 +942,12 @@
     <row r="17" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="2"/>
       <c r="B17" s="1" t="s">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="C17">
-        <v>4</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="D17" s="1"/>
       <c r="E17">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1028,10 +956,10 @@
     <row r="18" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="2"/>
       <c r="B18" s="1" t="s">
-        <v>26</v>
+        <v>5</v>
       </c>
       <c r="C18">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E18">
         <f t="shared" si="0"/>
@@ -1041,7 +969,7 @@
     <row r="19" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="2"/>
       <c r="B19" s="1" t="s">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="C19">
         <v>1</v>
@@ -1054,7 +982,7 @@
     <row r="20" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="2"/>
       <c r="B20" s="1" t="s">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="C20">
         <v>1</v>
@@ -1065,39 +993,40 @@
       </c>
     </row>
     <row r="21" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="2"/>
       <c r="B21" s="1" t="s">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="C21">
+        <v>1</v>
+      </c>
+      <c r="E21">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B22" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C22">
         <f>16+5</f>
         <v>21</v>
       </c>
-      <c r="D21">
+      <c r="D22">
         <v>1.5</v>
       </c>
-      <c r="E21">
+      <c r="E22">
         <f t="shared" si="0"/>
         <v>31.5</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C22">
-        <v>16</v>
-      </c>
-      <c r="E22">
-        <f t="shared" si="0"/>
-        <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B23" s="1" t="s">
-        <v>31</v>
+        <v>10</v>
       </c>
       <c r="C23">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="E23">
         <f t="shared" si="0"/>
@@ -1106,10 +1035,10 @@
     </row>
     <row r="24" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B24" s="1" t="s">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="C24">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="E24">
         <f t="shared" si="0"/>
@@ -1118,10 +1047,10 @@
     </row>
     <row r="25" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B25" s="1" t="s">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="C25">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="E25">
         <f t="shared" si="0"/>
@@ -1130,24 +1059,24 @@
     </row>
     <row r="26" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B26" s="1" t="s">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="C26">
+        <v>2</v>
+      </c>
+      <c r="E26">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B27" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C27">
         <f>16+5+1</f>
         <v>22</v>
       </c>
-      <c r="E26">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B27" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="C27">
-        <v>1</v>
-      </c>
       <c r="E27">
         <f t="shared" si="0"/>
         <v>0</v>
@@ -1155,7 +1084,7 @@
     </row>
     <row r="28" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B28" s="1" t="s">
-        <v>36</v>
+        <v>15</v>
       </c>
       <c r="C28">
         <v>1</v>
@@ -1167,10 +1096,10 @@
     </row>
     <row r="29" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B29" s="1" t="s">
-        <v>37</v>
+        <v>16</v>
       </c>
       <c r="C29">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="E29">
         <f t="shared" si="0"/>
@@ -1179,10 +1108,10 @@
     </row>
     <row r="30" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B30" s="1" t="s">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="C30">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="E30">
         <f t="shared" si="0"/>
@@ -1191,10 +1120,10 @@
     </row>
     <row r="31" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B31" s="1" t="s">
-        <v>39</v>
+        <v>18</v>
       </c>
       <c r="C31">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E31">
         <f t="shared" si="0"/>
@@ -1203,51 +1132,53 @@
     </row>
     <row r="32" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B32" s="1" t="s">
-        <v>40</v>
+        <v>19</v>
       </c>
       <c r="C32">
+        <v>9</v>
+      </c>
+      <c r="E32">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B33" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C33">
         <v>4</v>
       </c>
-      <c r="D32">
+      <c r="D33">
         <v>0.40749999999999997</v>
       </c>
-      <c r="E32">
+      <c r="E33">
         <f t="shared" si="0"/>
         <v>1.63</v>
       </c>
     </row>
-    <row r="33" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="C33">
+    <row r="34" spans="1:5" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C34">
         <v>7</v>
       </c>
-      <c r="D33">
+      <c r="D34">
         <v>345.15</v>
       </c>
-      <c r="E33">
+      <c r="E34">
         <f t="shared" si="0"/>
         <v>2416.0499999999997</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="2"/>
-      <c r="B34" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E34">
-        <f t="shared" si="0"/>
-        <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="2"/>
       <c r="B35" s="1" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="E35">
         <f t="shared" si="0"/>
@@ -1257,7 +1188,7 @@
     <row r="36" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="2"/>
       <c r="B36" s="1" t="s">
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="E36">
         <f t="shared" si="0"/>
@@ -1267,7 +1198,7 @@
     <row r="37" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="2"/>
       <c r="B37" s="1" t="s">
-        <v>46</v>
+        <v>24</v>
       </c>
       <c r="E37">
         <f t="shared" si="0"/>
@@ -1275,8 +1206,9 @@
       </c>
     </row>
     <row r="38" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="2"/>
       <c r="B38" s="1" t="s">
-        <v>47</v>
+        <v>25</v>
       </c>
       <c r="E38">
         <f t="shared" si="0"/>
@@ -1285,41 +1217,50 @@
     </row>
     <row r="39" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B39" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="C39">
-        <v>1</v>
-      </c>
-      <c r="D39">
-        <v>33.4</v>
+        <v>26</v>
       </c>
       <c r="E39">
         <f t="shared" si="0"/>
-        <v>33.4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B40" s="1" t="s">
-        <v>49</v>
+        <v>27</v>
       </c>
       <c r="C40">
         <v>1</v>
       </c>
       <c r="D40">
+        <v>33.4</v>
+      </c>
+      <c r="E40">
+        <f t="shared" si="0"/>
+        <v>33.4</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B41" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C41">
+        <v>1</v>
+      </c>
+      <c r="D41">
         <v>52</v>
       </c>
-      <c r="E40">
+      <c r="E41">
         <f t="shared" si="0"/>
         <v>52</v>
       </c>
     </row>
-    <row r="42" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D42" t="s">
-        <v>50</v>
-      </c>
-      <c r="E42">
-        <f>SUM(E2:E40)</f>
-        <v>2958.58</v>
+    <row r="45" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D45" t="s">
+        <v>29</v>
+      </c>
+      <c r="E45">
+        <f>SUM(E2:E41)</f>
+        <v>3028.1899999999996</v>
       </c>
     </row>
   </sheetData>

</xml_diff>